<commit_message>
Finished statistical analysis. Added is_doi to statistical analysis. Added p values (still need to be formatted) and age-citations relationship to index.qmd. Next steps: Finish verifying counts across vars script, plots prep, plots and statistical analysis. Update is_doi in all_sources and 1 more non-matched sample to metadata and all_sources
</commit_message>
<xml_diff>
--- a/summarise_distinct_matches.xlsx
+++ b/summarise_distinct_matches.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AVIHAY\git\DCC-v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{E437BC66-5941-4181-998C-1380A7BFA348}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25EE7D97-39FE-496B-BF36-7B158D94226C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="summarise_distinct_matches" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="165">
   <si>
     <t>file</t>
   </si>
@@ -523,7 +523,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -660,7 +660,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -848,12 +848,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1019,11 +1013,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1387,7 +1380,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:E284"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4196,323 +4189,407 @@
         <v>7</v>
       </c>
     </row>
-    <row r="200" spans="1:4" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A200" s="3" t="s">
+    <row r="200" spans="1:4" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B200" s="3">
+      <c r="B200" s="2">
         <v>531</v>
       </c>
-      <c r="C200" s="3" t="s">
+      <c r="C200" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D200" s="3" t="s">
+      <c r="D200" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A201" s="2" t="s">
+      <c r="A201" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B201">
         <v>205</v>
       </c>
+      <c r="C201" t="s">
+        <v>6</v>
+      </c>
       <c r="D201" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A202" s="2" t="s">
+      <c r="A202" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B202">
         <v>583</v>
       </c>
+      <c r="C202" t="s">
+        <v>6</v>
+      </c>
       <c r="D202" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A203" s="2" t="s">
+      <c r="A203" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B203">
         <v>585</v>
       </c>
+      <c r="C203" t="s">
+        <v>6</v>
+      </c>
       <c r="D203" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A204" s="2" t="s">
+      <c r="A204" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B204">
         <v>120</v>
       </c>
+      <c r="C204" t="s">
+        <v>6</v>
+      </c>
       <c r="D204" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A205" s="2" t="s">
+      <c r="A205" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B205">
         <v>121</v>
       </c>
+      <c r="C205" t="s">
+        <v>6</v>
+      </c>
       <c r="D205" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A206" s="2" t="s">
+      <c r="A206" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B206">
         <v>122</v>
       </c>
+      <c r="C206" t="s">
+        <v>6</v>
+      </c>
       <c r="D206" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A207" s="2" t="s">
+      <c r="A207" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B207">
         <v>129</v>
       </c>
+      <c r="C207" t="s">
+        <v>6</v>
+      </c>
       <c r="D207" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A208" s="2" t="s">
+      <c r="A208" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B208">
         <v>130</v>
       </c>
+      <c r="C208" t="s">
+        <v>6</v>
+      </c>
       <c r="D208" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A209" s="2" t="s">
+      <c r="A209" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B209">
         <v>131</v>
       </c>
+      <c r="C209" t="s">
+        <v>6</v>
+      </c>
       <c r="D209" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A210" s="2" t="s">
+      <c r="A210" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B210">
         <v>176</v>
       </c>
+      <c r="C210" t="s">
+        <v>6</v>
+      </c>
       <c r="D210" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A211" s="2" t="s">
+      <c r="A211" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B211">
         <v>177</v>
       </c>
+      <c r="C211" t="s">
+        <v>6</v>
+      </c>
       <c r="D211" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A212" s="2" t="s">
+      <c r="A212" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B212">
         <v>178</v>
       </c>
+      <c r="C212" t="s">
+        <v>6</v>
+      </c>
       <c r="D212" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A213" s="2" t="s">
+      <c r="A213" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B213">
         <v>225</v>
       </c>
+      <c r="C213" t="s">
+        <v>6</v>
+      </c>
       <c r="D213" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A214" s="2" t="s">
+      <c r="A214" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B214">
         <v>235</v>
       </c>
+      <c r="C214" t="s">
+        <v>6</v>
+      </c>
       <c r="D214" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A215" s="2" t="s">
+      <c r="A215" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B215">
         <v>243</v>
       </c>
+      <c r="C215" t="s">
+        <v>6</v>
+      </c>
       <c r="D215" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A216" s="2" t="s">
+      <c r="A216" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B216">
         <v>253</v>
       </c>
+      <c r="C216" t="s">
+        <v>6</v>
+      </c>
       <c r="D216" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A217" s="2" t="s">
+      <c r="A217" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B217">
         <v>254</v>
       </c>
+      <c r="C217" t="s">
+        <v>6</v>
+      </c>
       <c r="D217" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A218" s="2" t="s">
+      <c r="A218" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B218">
         <v>255</v>
       </c>
+      <c r="C218" t="s">
+        <v>6</v>
+      </c>
       <c r="D218" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A219" s="2" t="s">
+      <c r="A219" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B219">
         <v>284</v>
       </c>
+      <c r="C219" t="s">
+        <v>6</v>
+      </c>
       <c r="D219" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A220" s="2" t="s">
+      <c r="A220" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B220">
         <v>321</v>
       </c>
+      <c r="C220" t="s">
+        <v>6</v>
+      </c>
       <c r="D220" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A221" s="2" t="s">
+      <c r="A221" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B221">
         <v>338</v>
       </c>
+      <c r="C221" t="s">
+        <v>6</v>
+      </c>
       <c r="D221" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A222" s="2" t="s">
+      <c r="A222" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B222">
         <v>357</v>
       </c>
+      <c r="C222" t="s">
+        <v>6</v>
+      </c>
       <c r="D222" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A223" s="2" t="s">
+      <c r="A223" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B223">
         <v>375</v>
       </c>
+      <c r="C223" t="s">
+        <v>6</v>
+      </c>
       <c r="D223" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A224" s="2" t="s">
+      <c r="A224" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B224">
         <v>393</v>
       </c>
+      <c r="C224" t="s">
+        <v>6</v>
+      </c>
       <c r="D224" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A225" s="2" t="s">
+      <c r="A225" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B225">
         <v>509</v>
       </c>
+      <c r="C225" t="s">
+        <v>6</v>
+      </c>
       <c r="D225" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A226" s="2" t="s">
+      <c r="A226" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B226">
         <v>512</v>
       </c>
+      <c r="C226" t="s">
+        <v>6</v>
+      </c>
       <c r="D226" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A227" s="2" t="s">
+      <c r="A227" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B227">
         <v>531</v>
       </c>
+      <c r="C227" t="s">
+        <v>6</v>
+      </c>
       <c r="D227" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="228" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A228" s="2" t="s">
+      <c r="A228" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B228">
         <v>579</v>
+      </c>
+      <c r="C228" t="s">
+        <v>6</v>
       </c>
       <c r="D228" t="s">
         <v>69</v>
@@ -4872,348 +4949,441 @@
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A254" s="2" t="s">
+      <c r="A254" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B254">
         <v>107</v>
       </c>
+      <c r="C254" t="s">
+        <v>6</v>
+      </c>
       <c r="D254" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A255" s="2" t="s">
+      <c r="A255" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B255">
         <v>161</v>
       </c>
+      <c r="C255" t="s">
+        <v>6</v>
+      </c>
       <c r="D255" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A256" s="2" t="s">
+      <c r="A256" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B256">
         <v>164</v>
       </c>
+      <c r="C256" t="s">
+        <v>6</v>
+      </c>
       <c r="D256" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A257" s="2" t="s">
+      <c r="A257" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B257">
         <v>167</v>
       </c>
+      <c r="C257" t="s">
+        <v>6</v>
+      </c>
       <c r="D257" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A258" s="2" t="s">
+      <c r="A258" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B258">
         <v>170</v>
       </c>
+      <c r="C258" t="s">
+        <v>6</v>
+      </c>
       <c r="D258" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A259" s="2" t="s">
+      <c r="A259" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B259">
         <v>173</v>
       </c>
+      <c r="C259" t="s">
+        <v>6</v>
+      </c>
       <c r="D259" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A260" s="2" t="s">
+      <c r="A260" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B260">
         <v>176</v>
       </c>
+      <c r="C260" t="s">
+        <v>6</v>
+      </c>
       <c r="D260" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A261" s="2" t="s">
+      <c r="A261" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B261">
         <v>179</v>
       </c>
+      <c r="C261" t="s">
+        <v>6</v>
+      </c>
       <c r="D261" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A262" s="2" t="s">
+      <c r="A262" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B262">
         <v>183</v>
       </c>
+      <c r="C262" t="s">
+        <v>6</v>
+      </c>
       <c r="D262" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A263" s="2" t="s">
+      <c r="A263" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B263">
         <v>186</v>
       </c>
+      <c r="C263" t="s">
+        <v>6</v>
+      </c>
       <c r="D263" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A264" s="2" t="s">
+      <c r="A264" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B264">
         <v>190</v>
       </c>
+      <c r="C264" t="s">
+        <v>6</v>
+      </c>
       <c r="D264" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A265" s="2" t="s">
+      <c r="A265" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B265">
         <v>198</v>
       </c>
+      <c r="C265" t="s">
+        <v>6</v>
+      </c>
       <c r="D265" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A266" s="2" t="s">
+      <c r="A266" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B266">
         <v>206</v>
       </c>
+      <c r="C266" t="s">
+        <v>6</v>
+      </c>
       <c r="D266" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A267" s="2" t="s">
+      <c r="A267" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B267">
         <v>212</v>
       </c>
+      <c r="C267" t="s">
+        <v>6</v>
+      </c>
       <c r="D267" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A268" s="2" t="s">
+      <c r="A268" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B268">
         <v>215</v>
       </c>
+      <c r="C268" t="s">
+        <v>6</v>
+      </c>
       <c r="D268" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A269" s="2" t="s">
+      <c r="A269" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B269">
         <v>218</v>
       </c>
+      <c r="C269" t="s">
+        <v>6</v>
+      </c>
       <c r="D269" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A270" s="2" t="s">
+      <c r="A270" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B270">
         <v>222</v>
       </c>
+      <c r="C270" t="s">
+        <v>6</v>
+      </c>
       <c r="D270" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A271" s="2" t="s">
+      <c r="A271" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B271">
         <v>225</v>
       </c>
+      <c r="C271" t="s">
+        <v>6</v>
+      </c>
       <c r="D271" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A272" s="2" t="s">
+      <c r="A272" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B272">
         <v>228</v>
       </c>
+      <c r="C272" t="s">
+        <v>6</v>
+      </c>
       <c r="D272" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A273" s="2" t="s">
+      <c r="A273" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B273">
         <v>232</v>
       </c>
+      <c r="C273" t="s">
+        <v>6</v>
+      </c>
       <c r="D273" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A274" s="2" t="s">
+      <c r="A274" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B274">
         <v>235</v>
       </c>
+      <c r="C274" t="s">
+        <v>6</v>
+      </c>
       <c r="D274" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A275" s="2" t="s">
+      <c r="A275" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B275">
         <v>238</v>
       </c>
+      <c r="C275" t="s">
+        <v>6</v>
+      </c>
       <c r="D275" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A276" s="2" t="s">
+      <c r="A276" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B276">
         <v>241</v>
       </c>
+      <c r="C276" t="s">
+        <v>6</v>
+      </c>
       <c r="D276" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A277" s="2" t="s">
+      <c r="A277" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B277">
         <v>245</v>
       </c>
+      <c r="C277" t="s">
+        <v>6</v>
+      </c>
       <c r="D277" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A278" s="2" t="s">
+      <c r="A278" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B278">
         <v>248</v>
       </c>
+      <c r="C278" t="s">
+        <v>6</v>
+      </c>
       <c r="D278" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A279" s="2" t="s">
+      <c r="A279" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B279">
         <v>251</v>
       </c>
+      <c r="C279" t="s">
+        <v>6</v>
+      </c>
       <c r="D279" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A280" s="2" t="s">
+      <c r="A280" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B280">
         <v>254</v>
       </c>
+      <c r="C280" t="s">
+        <v>6</v>
+      </c>
       <c r="D280" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A281" s="2" t="s">
+      <c r="A281" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B281">
         <v>264</v>
       </c>
+      <c r="C281" t="s">
+        <v>6</v>
+      </c>
       <c r="D281" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A282" s="2" t="s">
+      <c r="A282" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B282">
         <v>267</v>
       </c>
+      <c r="C282" t="s">
+        <v>6</v>
+      </c>
       <c r="D282" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A283" s="2" t="s">
+      <c r="A283" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B283">
         <v>270</v>
       </c>
+      <c r="C283" t="s">
+        <v>6</v>
+      </c>
       <c r="D283" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A284" s="2" t="s">
+      <c r="A284" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B284">
         <v>273</v>
       </c>
+      <c r="C284" t="s">
+        <v>6</v>
+      </c>
       <c r="D284" t="s">
         <v>162</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E284">
+  <autoFilter ref="A1:E284" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="0">
       <colorFilter dxfId="0"/>
     </filterColumn>

</xml_diff>